<commit_message>
update ihe careteam 4e57f094665651845992f8ad93cadfa1b3366def
</commit_message>
<xml_diff>
--- a/nr-test-template-2/ig/StructureDefinition-cds-ihe-careteam.xlsx
+++ b/nr-test-template-2/ig/StructureDefinition-cds-ihe-careteam.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-28T13:58:36+00:00</t>
+    <t>2026-05-28T14:14:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -811,8 +811,7 @@
     <t>CareTeam.status</t>
   </si>
   <si>
-    <t>Statut du cercle de soins.
- valeurs autorisées : proposed | active | suspended | inactive | entered-in-error</t>
+    <t>Statut du cercle de soins. valeurs autorisées : proposed | active | suspended | inactive | entered-in-error</t>
   </si>
   <si>
     <t>Indicates the current state of the care team.</t>

</xml_diff>